<commit_message>
Update Excel/CSV with zero-padded codes + new collection names
</commit_message>
<xml_diff>
--- a/exhibition-links.xlsx
+++ b/exhibition-links.xlsx
@@ -466,14 +466,14 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -484,7 +484,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Code No.</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -494,7 +494,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Installation Location</t>
+          <t>Collection</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -514,12 +514,12 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Size (cm)</t>
+          <t>Size</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>NFC Link URL</t>
+          <t>Link URL</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>1/JM</t>
+          <t>01/JM</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Podium / Stage Wings</t>
+          <t>Heritage Collection</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>https://beyondtenun.vercel.app/record/1%2FJM</t>
+          <t>https://beyondtenun.vercel.app/record/01%2FJM</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2/GW</t>
+          <t>02/GW</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -584,7 +584,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Rear Wall / Long Side Wall</t>
+          <t>Gallery</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>https://beyondtenun.vercel.app/record/2%2FGW</t>
+          <t>https://beyondtenun.vercel.app/record/02%2FGW</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>3/GW</t>
+          <t>03/GW</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Rear Wall / Long Side Wall</t>
+          <t>Gallery</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>https://beyondtenun.vercel.app/record/3%2FGW</t>
+          <t>https://beyondtenun.vercel.app/record/03%2FGW</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>4/TM</t>
+          <t>04/TM</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Registration Table</t>
+          <t>Weave Archive</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>https://beyondtenun.vercel.app/record/4%2FTM</t>
+          <t>https://beyondtenun.vercel.app/record/04%2FTM</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>5/GW</t>
+          <t>05/GW</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Rear Wall / Long Side Wall</t>
+          <t>Gallery</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>https://beyondtenun.vercel.app/record/5%2FGW</t>
+          <t>https://beyondtenun.vercel.app/record/05%2FGW</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>6/GW</t>
+          <t>06/GW</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Rear Wall / Long Side Wall</t>
+          <t>Gallery</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>https://beyondtenun.vercel.app/record/6%2FGW</t>
+          <t>https://beyondtenun.vercel.app/record/06%2FGW</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>7/TM</t>
+          <t>07/TM</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Registration Table</t>
+          <t>Weave Archive</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>https://beyondtenun.vercel.app/record/7%2FTM</t>
+          <t>https://beyondtenun.vercel.app/record/07%2FTM</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Podium / Stage Wings</t>
+          <t>Heritage Collection</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>8/TM</t>
+          <t>08/TM</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Registration Table</t>
+          <t>Weave Archive</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>https://beyondtenun.vercel.app/record/8%2FTM</t>
+          <t>https://beyondtenun.vercel.app/record/08%2FTM</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>9/TM</t>
+          <t>09/TM</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Registration Table</t>
+          <t>Weave Archive</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>https://beyondtenun.vercel.app/record/9%2FTM</t>
+          <t>https://beyondtenun.vercel.app/record/09%2FTM</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Registration Table</t>
+          <t>Weave Archive</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Registration Table</t>
+          <t>Weave Archive</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Registration Table</t>
+          <t>Weave Archive</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Rear Wall / Long Side Wall</t>
+          <t>Gallery</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Rear Wall / Long Side Wall</t>
+          <t>Gallery</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Podium / Stage Wings</t>
+          <t>Heritage Collection</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Podium / Stage Wings</t>
+          <t>Heritage Collection</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Rear Wall / Long Side Wall</t>
+          <t>Gallery</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Rear Wall / Long Side Wall</t>
+          <t>Gallery</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Rear Wall / Long Side Wall</t>
+          <t>Gallery</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Rear Wall / Long Side Wall</t>
+          <t>Gallery</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Stage: Super Long (Not for Sale)</t>
+          <t>Not for Sale</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Stage: Super Long (Not for Sale)</t>
+          <t>Not for Sale</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Stage: Super Long (Not for Sale)</t>
+          <t>Not for Sale</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Stage: Super Long (Not for Sale)</t>
+          <t>Not for Sale</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Stage: Super Long (Not for Sale)</t>
+          <t>Not for Sale</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Stage: Super Long (Not for Sale)</t>
+          <t>Not for Sale</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Registration Table</t>
+          <t>Weave Archive</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Stage Wings / Side Partitions / Registration Table</t>
+          <t>Weave Archive</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1858,7 +1858,7 @@
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -1877,7 +1877,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Gallery Wall</t>
+          <t>Gallery</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
@@ -1887,7 +1887,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Jejak Masters</t>
+          <t>Heritage Collection</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
@@ -1907,7 +1907,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Tenun Masters</t>
+          <t>Weave Archive</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">

</xml_diff>

<commit_message>
Add full cloth data from TORAJAMELO Handwoven List sheet
The xlsx is now the source of truth for origin, technique, material and
size.  Per record:
  · Origin, Technique, Material (sentence-cased, " - " -> ", "),
    Size with a proper multiplication sign, and a new "Displayed at"
    attribute carrying the sheet's Installation Location
  · names cleaned of the code suffix the sheet appends ("Tais Feto
    Biboki/GW" -> "Tais Feto Biboki")
  · sorted in exhibition order

UI: "Displayed at" shown in the Material tab on the record page.
Excel/CSV export regenerated with the Displayed at column.
01/JM falls back to the placeholder photo (no photo supplied).
</commit_message>
<xml_diff>
--- a/exhibition-links.xlsx
+++ b/exhibition-links.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Exhibition Links'!$A$1:$I$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Exhibition Links'!$A$1:$J$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,9 @@
       <color rgb="00AE1800"/>
       <sz val="10"/>
       <u val="single"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -85,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -97,6 +100,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -462,18 +466,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -514,10 +519,15 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Size</t>
+          <t>Size (cm)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Displayed at</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Link URL</t>
         </is>
@@ -534,7 +544,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Gringsing Tenganan / Gringsing Wayang</t>
+          <t>Gringsing Tenganan, Gringsing Wayang</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -554,7 +564,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Handspun cotton, natural dyes</t>
+          <t>Handspun Cotton, natural dyes</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -562,7 +572,12 @@
           <t>198 × 54</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Podium</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>https://beyondtenun.vercel.app/record/01%2FJM</t>
         </is>
@@ -607,7 +622,12 @@
           <t>137 × 57</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Stage : Left &amp; Right (portable partitions)</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>https://beyondtenun.vercel.app/record/02%2FGW</t>
         </is>
@@ -639,7 +659,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Warp ikat</t>
+          <t>Warp Ikat</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -652,7 +672,12 @@
           <t>180 × 97</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Stage : Left &amp; Right (portable partitions)</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>https://beyondtenun.vercel.app/record/03%2FGW</t>
         </is>
@@ -697,7 +722,12 @@
           <t>182 × 74</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Stage : Left &amp; Right (portable partitions)</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>https://beyondtenun.vercel.app/record/04%2FTM</t>
         </is>
@@ -734,7 +764,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Cotton</t>
+          <t>Cotton, chemical dyes</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -742,7 +772,12 @@
           <t>174 × 58.5</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Stage : Left &amp; Right (portable partitions)</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>https://beyondtenun.vercel.app/record/05%2FGW</t>
         </is>
@@ -779,7 +814,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Cotton</t>
+          <t>Cotton, chemical dyes</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -787,7 +822,12 @@
           <t>118 × 64</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Stage : Left &amp; Right (portable partitions)</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>https://beyondtenun.vercel.app/record/06%2FGW</t>
         </is>
@@ -824,7 +864,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Cotton</t>
+          <t>Cotton, chemical dyes</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -832,7 +872,12 @@
           <t>144 × 65</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Stage : Left &amp; Right (portable partitions)</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>https://beyondtenun.vercel.app/record/07%2FTM</t>
         </is>
@@ -844,34 +889,47 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>21/JM</t>
+          <t>08/TM</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Tapis Inuh Lampung</t>
+          <t>Sandung, Ruit, Perahu</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Heritage Collection</t>
+          <t>Weave Archive</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Lampung/Sumatera Selatan</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
+          <t>Sintang/Kalimantan Barat</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Warp ikat</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Cotton, chemical dyes</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>120 × 130</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/21%2FJM</t>
+          <t>134 × 56</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Portable Partitions on the side</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/08%2FTM</t>
         </is>
       </c>
     </row>
@@ -881,12 +939,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>08/TM</t>
+          <t>09/TM</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Sandung, Ruit, Perahu</t>
+          <t>Ikat Langa</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -896,7 +954,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Sintang/Kalimantan Barat</t>
+          <t>Bajawa/NTT</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -906,17 +964,22 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Cotton, chemical dyes</t>
+          <t>Cotton, natural dyes</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>134 × 56</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/08%2FTM</t>
+          <t>150 × 56</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Portable Partitions on the side</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/09%2FTM</t>
         </is>
       </c>
     </row>
@@ -926,12 +989,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>09/TM</t>
+          <t>10/TM</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Ikat Langa</t>
+          <t>Gringsing</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -941,27 +1004,32 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Bajawa/NTT</t>
+          <t>Karangasem/Bali</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Warp ikat</t>
+          <t>Double ikat</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Cotton, natural dyes</t>
+          <t>Handspun Cotton, natural dyes</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>150 × 56</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/09%2FTM</t>
+          <t>236 × 43</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Portable Partitions on the side</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/10%2FTM</t>
         </is>
       </c>
     </row>
@@ -971,12 +1039,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>10/TM</t>
+          <t>11/TM</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Gringsing</t>
+          <t>Penetoten</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -986,27 +1054,32 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Karangasem/Bali</t>
+          <t>Lembata/NTT</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Double ikat</t>
+          <t>Supplementary warp</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Handspun cotton, natural dyes</t>
+          <t>Cotton, chemical dyes</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>236 × 43</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/10%2FTM</t>
+          <t>189 × 68</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Portable Partitions on the side</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/11%2FTM</t>
         </is>
       </c>
     </row>
@@ -1016,12 +1089,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>11/TM</t>
+          <t>12/TM</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Penetoten</t>
+          <t>Songket</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1031,27 +1104,32 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Lembata/NTT</t>
+          <t>Sukarara/NTB</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Supplementary warp</t>
+          <t>Supplementary weft</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Cotton, chemical dyes</t>
+          <t>Cotton-Natural dyes</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>189 × 68</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/11%2FTM</t>
+          <t>183 × 106</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Portable Partitions on the side</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/12%2FTM</t>
         </is>
       </c>
     </row>
@@ -1061,42 +1139,47 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>12/TM</t>
+          <t>13/GW</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Songket</t>
+          <t>Lau Witikau</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Weave Archive</t>
+          <t>Gallery</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Sukarara/NTB</t>
+          <t>Sumba Timur/NTT</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Supplementary weft</t>
+          <t>Plain weave</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Cotton, natural dyes</t>
+          <t>Cotton, nassa shellls, beads</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>183 × 106</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/12%2FTM</t>
+          <t>97 × 54</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Portable Partitions on the side</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/13%2FGW</t>
         </is>
       </c>
     </row>
@@ -1106,12 +1189,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>13/GW</t>
+          <t>14/GW</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Lau Witikau</t>
+          <t>Ei Worapi</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1121,27 +1204,32 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Sumba Timur/NTT</t>
+          <t>Sawu/NTT</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Plain weave</t>
+          <t>Warp ikat</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Cotton, Nassa shells, beads</t>
+          <t>Cotton, natural dyes</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>97 × 54</t>
-        </is>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/13%2FGW</t>
+          <t>160 × 58</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Portable Partitions on the side</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/14%2FGW</t>
         </is>
       </c>
     </row>
@@ -1151,22 +1239,22 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>14/GW</t>
+          <t>15/JM</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Ei Worapi</t>
+          <t>Kewatek Nai Telo</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Gallery</t>
+          <t>Heritage Collection</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Sawu/NTT</t>
+          <t>Lembata/NTT</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1176,17 +1264,22 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Cotton, natural dyes</t>
+          <t>Handspun Cotton, natural dyes</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>160 × 58</t>
-        </is>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/14%2FGW</t>
+          <t>180 × 78</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Portable Partitions on the side</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/15%2FJM</t>
         </is>
       </c>
     </row>
@@ -1196,12 +1289,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>15/JM</t>
+          <t>16/JM</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Kewatek Nai Telo</t>
+          <t>Amanuban</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1211,7 +1304,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Lembata/NTT</t>
+          <t>Timor Tengah Selatan (TTS)/NTT</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1221,17 +1314,22 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Handspun cotton, natural dyes</t>
+          <t>Cotton, mix dyes</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>180 × 78</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/15%2FJM</t>
+          <t>180 × 92</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Portable Partitions on the side</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/16%2FJM</t>
         </is>
       </c>
     </row>
@@ -1241,22 +1339,22 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>16/JM</t>
+          <t>17/GW</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Amanuban</t>
+          <t>Hanggi</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Heritage Collection</t>
+          <t>Gallery</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Timor Tengah Selatan (TTS)/NTT</t>
+          <t>Sumba Barat/NTT</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1266,17 +1364,22 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Cotton, mix dyes</t>
+          <t>Cotton, chemical dyes</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>180 × 92</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/16%2FJM</t>
+          <t>252 × 112.5</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Rear Wall</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/17%2FGW</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1422,12 @@
           <t>232 × 123.5</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Rear Wall</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
         <is>
           <t>https://beyondtenun.vercel.app/record/18%2FGW</t>
         </is>
@@ -1331,12 +1439,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>17/GW</t>
+          <t>19/GW</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Hanggi</t>
+          <t>Rohubangi - A</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1346,27 +1454,32 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Sumba Barat/NTT</t>
+          <t>Sumba Timur/NTT</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Warp ikat</t>
+          <t>Supplementary warp</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Cotton, chemical dyes</t>
+          <t>Cotton, natural dyes</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>252 × 112.5</t>
-        </is>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/17%2FGW</t>
+          <t>448 × 48.5</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Long Side Wall</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/19%2FGW</t>
         </is>
       </c>
     </row>
@@ -1376,12 +1489,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>19/GW</t>
+          <t>20/GW</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Rohubangi - A</t>
+          <t>Rohubangi - B</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1401,17 +1514,22 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Cotton</t>
+          <t>Cotton, chemical dyes</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>448 × 48.5</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/19%2FGW</t>
+          <t>530 × 37</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Long Side Wall</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/20%2FGW</t>
         </is>
       </c>
     </row>
@@ -1421,42 +1539,47 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>20/GW</t>
+          <t>21/JM</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Rohubangi - B</t>
+          <t>Tapis Inuh Lampung</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Gallery</t>
+          <t>Heritage Collection</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Sumba Timur/NTT</t>
+          <t>Lampung/Sumatera Selatan</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Supplementary warp</t>
+          <t>Ikat &amp; Emroidery</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Cotton</t>
+          <t>Cotton, mix dyes</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>530 × 37</t>
-        </is>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/20%2FGW</t>
+          <t>120 × 130</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Long Side Wall</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/21%2FJM</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1594,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Sakka - Maroon</t>
+          <t>Sakka-Maroon</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1499,7 +1622,12 @@
           <t>864 × 44</t>
         </is>
       </c>
-      <c r="I23" s="3" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Stage : Super Long (Not for Sale)</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
         <is>
           <t>https://beyondtenun.vercel.app/record/22%2FTM-NFS</t>
         </is>
@@ -1531,7 +1659,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Supplementary warp</t>
+          <t>Supplementary Warp</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1544,7 +1672,12 @@
           <t>960 × 46</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Stage : Super Long (Not for Sale)</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
         <is>
           <t>https://beyondtenun.vercel.app/record/23%2FTM-NFS</t>
         </is>
@@ -1576,7 +1709,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Supplementary warp</t>
+          <t>Supplementary Warp</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -1589,7 +1722,12 @@
           <t>1000 × 46</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Stage : Super Long (Not for Sale)</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
         <is>
           <t>https://beyondtenun.vercel.app/record/24%2FTM-NFS</t>
         </is>
@@ -1621,7 +1759,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Supplementary warp</t>
+          <t>Supplementary Warp</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -1634,7 +1772,12 @@
           <t>1010 × 48</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Stage : Super Long (Not for Sale)</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>https://beyondtenun.vercel.app/record/25%2FTM-NFS</t>
         </is>
@@ -1646,38 +1789,47 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>28/TM-NFS</t>
+          <t>26/TM</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Sakka - Red &amp; White (Long)</t>
+          <t>Pa'borong-Blue</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Not for Sale</t>
+          <t>Weave Archive</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Mamasa/Sulawesi Barat</t>
+          <t>Toraja/Sulawesi Selatan</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Supplementary warp</t>
+          <t>Plain weave</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Polyester</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/28%2FTM-NFS</t>
+          <t>Cotton, chemical dyes</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>340 × 55</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Registration Table</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/26%2FTM</t>
         </is>
       </c>
     </row>
@@ -1687,38 +1839,47 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>29/TM-NFS</t>
+          <t>27/TM</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Sakka - Red &amp; White (Short)</t>
+          <t>Pa'borong-Green</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Not for Sale</t>
+          <t>Weave Archive</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Mamasa/Sulawesi Barat</t>
+          <t>Toraja/Sulawesi Selatan</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Supplementary warp</t>
+          <t>Plain weave</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Wool</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/29%2FTM-NFS</t>
+          <t>Cotton, chemical dyes</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>352 × 55</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Registration Table</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/27%2FTM</t>
         </is>
       </c>
     </row>
@@ -1728,42 +1889,43 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>26/TM</t>
+          <t>28/TM-NFS</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Pa'borong - Blue</t>
+          <t>Sakka - Red&amp;White -Long</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Weave Archive</t>
+          <t>Not for Sale</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Toraja/Sulawesi Selatan</t>
+          <t>Mamasa/Sulawesi Barat</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Plain weave</t>
+          <t>Supplementary Warp</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Cotton, chemical dye</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>340 × 55</t>
-        </is>
-      </c>
-      <c r="I29" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/26%2FTM</t>
+          <t>Polyester</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Stage : Super Long (Not for Sale)</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/28%2FTM-NFS</t>
         </is>
       </c>
     </row>
@@ -1773,77 +1935,78 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>27/TM</t>
+          <t>29/TM-NFS</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Pa'borong - Green</t>
+          <t>Sakka - Red &amp;White - short</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Weave Archive</t>
+          <t>Not for Sale</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Toraja/Sulawesi Selatan</t>
+          <t>Mamasa/Sulawesi Barat</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Plain weave</t>
+          <t>Supplementary Warp</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Cotton, chemical dye</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>352 × 55</t>
-        </is>
-      </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>https://beyondtenun.vercel.app/record/27%2FTM</t>
+          <t>Woll</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Stage : Super Long (Not for Sale)</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>https://beyondtenun.vercel.app/record/29%2FTM-NFS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I30"/>
+  <autoFilter ref="A1:J30"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1855,7 +2018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1914,6 +2077,16 @@
         <v>9</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>